<commit_message>
WIP: Working Tab rename-at-completion (5-step statement pipeline canon)
Rick's ruling: the working tab is named 'Working Tab' from its birth at 32-1
until 33-3's final aggregate-and-format step, where it is RENAMED 'Income
Statement' as the amber tab flips to statement-purple — name and finality
earned together. Rick renamed the tab in Module-3-2.xlsx; Bike-Repair-End
carries the final names. Extractor invariant 10 expects 'Working Tab' exactly
and gains a name-hygiene audit (leading/trailing whitespace in a tab name
fails loudly). Pages 32-1/32-2/32-3/33-1 carry the working name; 33-3 gains
the christening beat; flow-check asserts pin both states.

Canon (generalizes to Module 4's statements): 1 set up a Working Tab;
2 copy the relevant ledger rows in; 3 sort in a sorter panel; 4 sorted rows
appear on the tab; 5 aggregate and format — the tab becomes the statement.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Bike-Repair-Source-Workbooks/Bike-Repair-Module-3-2.xlsx
+++ b/Bike-Repair-Source-Workbooks/Bike-Repair-Module-3-2.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ra1/Courses-Local/Instructional_Redesign_v2/Bike-Repair-Source-Workbooks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B58C71D-F2C4-1248-B3D6-D1B9521D6B37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D2D956A-56CA-604D-A245-0366D70A24B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5680" yWindow="2600" windowWidth="25820" windowHeight="27720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="39280" yWindow="700" windowWidth="25820" windowHeight="27720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Assets" sheetId="1" r:id="rId1"/>
     <sheet name="Liabilities" sheetId="2" r:id="rId2"/>
     <sheet name="Reasons" sheetId="3" r:id="rId3"/>
     <sheet name="Balance Sheet" sheetId="4" r:id="rId4"/>
-    <sheet name="Income Statement" sheetId="5" r:id="rId5"/>
+    <sheet name="Working Tab" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2781,7 +2781,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85BC05FC-8811-4645-B882-FEC1278A6A56}">
   <sheetPr>
-    <tabColor theme="7" tint="-0.249977111117893"/>
+    <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="B1:D46"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>

</xml_diff>